<commit_message>
chore: regenerate Excel templates with title column on payments
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/website/public/templates/invoices-template.xlsx
+++ b/website/public/templates/invoices-template.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D39"/>
+  <dimension ref="A1:D38"/>
   <cols>
     <col min="1" max="1" width="28.83203125" customWidth="1"/>
     <col min="2" max="2" width="44.83203125" customWidth="1"/>
@@ -676,41 +676,41 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>payment_method</v>
+        <v>quote_document_ref</v>
       </c>
       <c r="B25" t="str">
         <v>No</v>
       </c>
       <c r="C25" t="str">
-        <v>Payment method</v>
+        <v>Linked quote document_ref</v>
       </c>
       <c r="D25" t="str">
-        <v/>
+        <v>Must exist in DB</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>quote_document_ref</v>
+        <v>notes</v>
       </c>
       <c r="B26" t="str">
         <v>No</v>
       </c>
       <c r="C26" t="str">
-        <v>Linked quote document_ref</v>
+        <v>Notes</v>
       </c>
       <c r="D26" t="str">
-        <v>Must exist in DB</v>
+        <v/>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>notes</v>
+        <v>item_title</v>
       </c>
       <c r="B27" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="C27" t="str">
-        <v>Notes</v>
+        <v>Line item title</v>
       </c>
       <c r="D27" t="str">
         <v/>
@@ -718,123 +718,109 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>item_title</v>
+        <v>category</v>
       </c>
       <c r="B28" t="str">
-        <v>Yes</v>
+        <v>Yes, for payable</v>
       </c>
       <c r="C28" t="str">
-        <v>Line item title</v>
+        <v>Line item category</v>
       </c>
       <c r="D28" t="str">
-        <v/>
+        <v>materials, labor, subcontractor, equipment_rental, housing_food, other, software_licenses, partner_compensation, professional_services, other_sga</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>category</v>
+        <v>subtotal</v>
       </c>
       <c r="B29" t="str">
-        <v>Yes, for payable</v>
+        <v>Yes</v>
       </c>
       <c r="C29" t="str">
-        <v>Line item category</v>
+        <v>Line item subtotal (before IGV)</v>
       </c>
       <c r="D29" t="str">
-        <v>materials, labor, subcontractor, equipment_rental, housing_food, other, software_licenses, partner_compensation, professional_services, other_sga</v>
+        <v>Number, &gt; 0</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>subtotal</v>
+        <v>quantity</v>
       </c>
       <c r="B30" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="C30" t="str">
-        <v>Line item subtotal (before IGV)</v>
+        <v>Line item quantity</v>
       </c>
       <c r="D30" t="str">
-        <v>Number, &gt; 0</v>
+        <v>Number</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>quantity</v>
+        <v>unit_of_measure</v>
       </c>
       <c r="B31" t="str">
         <v>No</v>
       </c>
       <c r="C31" t="str">
-        <v>Line item quantity</v>
+        <v>Unit of measure</v>
       </c>
       <c r="D31" t="str">
-        <v>Number</v>
+        <v/>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>unit_of_measure</v>
+        <v>unit_price</v>
       </c>
       <c r="B32" t="str">
         <v>No</v>
       </c>
       <c r="C32" t="str">
-        <v>Unit of measure</v>
+        <v>Unit price</v>
       </c>
       <c r="D32" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="str">
-        <v>unit_price</v>
-      </c>
-      <c r="B33" t="str">
-        <v>No</v>
-      </c>
-      <c r="C33" t="str">
-        <v>Unit price</v>
-      </c>
-      <c r="D33" t="str">
         <v>Number</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>Notes:</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Notes:</v>
+        <v xml:space="preserve">  - Rows with the same document_ref are grouped into one invoice with multiple line items</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v xml:space="preserve">  - Rows with the same document_ref are grouped into one invoice with multiple line items</v>
+        <v xml:space="preserve">  - partner_name must match an entity tagged as "partner" in the database</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v xml:space="preserve">  - partner_name must match an entity tagged as "partner" in the database</v>
+        <v xml:space="preserve">  - Detracción only applies to PEN invoices</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v xml:space="preserve">  - Detracción only applies to PEN invoices</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="str">
         <v xml:space="preserve">  - Retención only applies to receivable invoices</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D39"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D38"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Y4"/>
+  <dimension ref="A1:X4"/>
   <cols>
     <col min="1" max="1" width="21.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -852,15 +838,14 @@
     <col min="14" max="14" width="19.83203125" customWidth="1"/>
     <col min="15" max="15" width="29.83203125" customWidth="1"/>
     <col min="16" max="16" width="16.83203125" customWidth="1"/>
-    <col min="17" max="17" width="16.83203125" customWidth="1"/>
-    <col min="18" max="18" width="27.83203125" customWidth="1"/>
-    <col min="19" max="19" width="12.83203125" customWidth="1"/>
-    <col min="20" max="20" width="17.83203125" customWidth="1"/>
-    <col min="21" max="21" width="40.83203125" customWidth="1"/>
-    <col min="22" max="22" width="33.83203125" customWidth="1"/>
-    <col min="23" max="23" width="20.83203125" customWidth="1"/>
-    <col min="24" max="24" width="17.83203125" customWidth="1"/>
-    <col min="25" max="25" width="12.83203125" customWidth="1"/>
+    <col min="17" max="17" width="27.83203125" customWidth="1"/>
+    <col min="18" max="18" width="12.83203125" customWidth="1"/>
+    <col min="19" max="19" width="17.83203125" customWidth="1"/>
+    <col min="20" max="20" width="40.83203125" customWidth="1"/>
+    <col min="21" max="21" width="33.83203125" customWidth="1"/>
+    <col min="22" max="22" width="20.83203125" customWidth="1"/>
+    <col min="23" max="23" width="17.83203125" customWidth="1"/>
+    <col min="24" max="24" width="12.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -913,30 +898,27 @@
         <v>retencion_rate</v>
       </c>
       <c r="Q1" t="str">
-        <v>payment_method</v>
+        <v>quote_document_ref</v>
       </c>
       <c r="R1" t="str">
-        <v>quote_document_ref</v>
+        <v>notes</v>
       </c>
       <c r="S1" t="str">
-        <v>notes</v>
+        <v>item_title</v>
       </c>
       <c r="T1" t="str">
-        <v>item_title</v>
+        <v>category</v>
       </c>
       <c r="U1" t="str">
-        <v>category</v>
+        <v>subtotal</v>
       </c>
       <c r="V1" t="str">
-        <v>subtotal</v>
+        <v>quantity</v>
       </c>
       <c r="W1" t="str">
-        <v>quantity</v>
+        <v>unit_of_measure</v>
       </c>
       <c r="X1" t="str">
-        <v>unit_of_measure</v>
-      </c>
-      <c r="Y1" t="str">
         <v>unit_price</v>
       </c>
     </row>
@@ -990,30 +972,27 @@
         <v>Retención rate</v>
       </c>
       <c r="Q2" t="str">
-        <v>Payment method</v>
+        <v>Linked quote document_ref</v>
       </c>
       <c r="R2" t="str">
-        <v>Linked quote document_ref</v>
+        <v>Notes</v>
       </c>
       <c r="S2" t="str">
-        <v>Notes</v>
+        <v>Line item title</v>
       </c>
       <c r="T2" t="str">
-        <v>Line item title</v>
+        <v>Line item category</v>
       </c>
       <c r="U2" t="str">
-        <v>Line item category</v>
+        <v>Line item subtotal (before IGV)</v>
       </c>
       <c r="V2" t="str">
-        <v>Line item subtotal (before IGV)</v>
+        <v>Line item quantity</v>
       </c>
       <c r="W2" t="str">
-        <v>Line item quantity</v>
+        <v>Unit of measure</v>
       </c>
       <c r="X2" t="str">
-        <v>Unit of measure</v>
-      </c>
-      <c r="Y2" t="str">
         <v>Unit price</v>
       </c>
     </row>
@@ -1067,30 +1046,27 @@
         <v>0.03</v>
       </c>
       <c r="Q3" t="str">
-        <v>transfer</v>
+        <v>COT-001</v>
       </c>
       <c r="R3" t="str">
-        <v>COT-001</v>
+        <v/>
       </c>
       <c r="S3" t="str">
-        <v/>
+        <v>Cement bags</v>
       </c>
       <c r="T3" t="str">
-        <v>Cement bags</v>
+        <v>materials</v>
       </c>
       <c r="U3" t="str">
-        <v>materials</v>
+        <v>5000.00</v>
       </c>
       <c r="V3" t="str">
-        <v>5000.00</v>
+        <v>200</v>
       </c>
       <c r="W3" t="str">
-        <v>200</v>
+        <v>bags</v>
       </c>
       <c r="X3" t="str">
-        <v>bags</v>
-      </c>
-      <c r="Y3" t="str">
         <v>25.00</v>
       </c>
     </row>
@@ -1144,36 +1120,33 @@
         <v/>
       </c>
       <c r="Q4" t="str">
-        <v/>
+        <v>Must exist in DB</v>
       </c>
       <c r="R4" t="str">
-        <v>Must exist in DB</v>
+        <v/>
       </c>
       <c r="S4" t="str">
         <v/>
       </c>
       <c r="T4" t="str">
-        <v/>
+        <v>materials, labor, subcontractor, equipment_rental, housing_food, other, software_licenses, partner_compensation, professional_services, other_sga</v>
       </c>
       <c r="U4" t="str">
-        <v>materials, labor, subcontractor, equipment_rental, housing_food, other, software_licenses, partner_compensation, professional_services, other_sga</v>
+        <v>Number, &gt; 0</v>
       </c>
       <c r="V4" t="str">
-        <v>Number, &gt; 0</v>
+        <v>Number</v>
       </c>
       <c r="W4" t="str">
-        <v>Number</v>
+        <v/>
       </c>
       <c r="X4" t="str">
-        <v/>
-      </c>
-      <c r="Y4" t="str">
         <v>Number</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Y4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:X4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: regenerate Excel import templates after quotes merge
Quotes template: added partner_name (required), category; removed igv_amount, total.
Invoices template: removed quote_document_ref column.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/website/public/templates/invoices-template.xlsx
+++ b/website/public/templates/invoices-template.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D38"/>
+  <dimension ref="A1:D37"/>
   <cols>
     <col min="1" max="1" width="28.83203125" customWidth="1"/>
     <col min="2" max="2" width="44.83203125" customWidth="1"/>
@@ -676,27 +676,27 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>quote_document_ref</v>
+        <v>notes</v>
       </c>
       <c r="B25" t="str">
         <v>No</v>
       </c>
       <c r="C25" t="str">
-        <v>Linked quote document_ref</v>
+        <v>Notes</v>
       </c>
       <c r="D25" t="str">
-        <v>Must exist in DB</v>
+        <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>notes</v>
+        <v>item_title</v>
       </c>
       <c r="B26" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="C26" t="str">
-        <v>Notes</v>
+        <v>Line item title</v>
       </c>
       <c r="D26" t="str">
         <v/>
@@ -704,123 +704,109 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>item_title</v>
+        <v>category</v>
       </c>
       <c r="B27" t="str">
-        <v>Yes</v>
+        <v>Yes, for payable</v>
       </c>
       <c r="C27" t="str">
-        <v>Line item title</v>
+        <v>Line item category</v>
       </c>
       <c r="D27" t="str">
-        <v/>
+        <v>materials, labor, subcontractor, equipment_rental, housing_food, other, software_licenses, partner_compensation, professional_services, other_sga</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>category</v>
+        <v>subtotal</v>
       </c>
       <c r="B28" t="str">
-        <v>Yes, for payable</v>
+        <v>Yes</v>
       </c>
       <c r="C28" t="str">
-        <v>Line item category</v>
+        <v>Line item subtotal (before IGV)</v>
       </c>
       <c r="D28" t="str">
-        <v>materials, labor, subcontractor, equipment_rental, housing_food, other, software_licenses, partner_compensation, professional_services, other_sga</v>
+        <v>Number, &gt; 0</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>subtotal</v>
+        <v>quantity</v>
       </c>
       <c r="B29" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="C29" t="str">
-        <v>Line item subtotal (before IGV)</v>
+        <v>Line item quantity</v>
       </c>
       <c r="D29" t="str">
-        <v>Number, &gt; 0</v>
+        <v>Number</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>quantity</v>
+        <v>unit_of_measure</v>
       </c>
       <c r="B30" t="str">
         <v>No</v>
       </c>
       <c r="C30" t="str">
-        <v>Line item quantity</v>
+        <v>Unit of measure</v>
       </c>
       <c r="D30" t="str">
-        <v>Number</v>
+        <v/>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>unit_of_measure</v>
+        <v>unit_price</v>
       </c>
       <c r="B31" t="str">
         <v>No</v>
       </c>
       <c r="C31" t="str">
-        <v>Unit of measure</v>
+        <v>Unit price</v>
       </c>
       <c r="D31" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="str">
-        <v>unit_price</v>
-      </c>
-      <c r="B32" t="str">
-        <v>No</v>
-      </c>
-      <c r="C32" t="str">
-        <v>Unit price</v>
-      </c>
-      <c r="D32" t="str">
         <v>Number</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>Notes:</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Notes:</v>
+        <v xml:space="preserve">  - Rows with the same document_ref are grouped into one invoice with multiple line items</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v xml:space="preserve">  - Rows with the same document_ref are grouped into one invoice with multiple line items</v>
+        <v xml:space="preserve">  - partner_name must match an entity tagged as "partner" in the database</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v xml:space="preserve">  - partner_name must match an entity tagged as "partner" in the database</v>
+        <v xml:space="preserve">  - Detracción only applies to PEN invoices</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v xml:space="preserve">  - Detracción only applies to PEN invoices</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="str">
         <v xml:space="preserve">  - Retención only applies to receivable invoices</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D38"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D37"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:X4"/>
+  <dimension ref="A1:W4"/>
   <cols>
     <col min="1" max="1" width="21.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -838,14 +824,13 @@
     <col min="14" max="14" width="19.83203125" customWidth="1"/>
     <col min="15" max="15" width="29.83203125" customWidth="1"/>
     <col min="16" max="16" width="16.83203125" customWidth="1"/>
-    <col min="17" max="17" width="27.83203125" customWidth="1"/>
-    <col min="18" max="18" width="12.83203125" customWidth="1"/>
-    <col min="19" max="19" width="17.83203125" customWidth="1"/>
-    <col min="20" max="20" width="40.83203125" customWidth="1"/>
-    <col min="21" max="21" width="33.83203125" customWidth="1"/>
-    <col min="22" max="22" width="20.83203125" customWidth="1"/>
-    <col min="23" max="23" width="17.83203125" customWidth="1"/>
-    <col min="24" max="24" width="12.83203125" customWidth="1"/>
+    <col min="17" max="17" width="12.83203125" customWidth="1"/>
+    <col min="18" max="18" width="17.83203125" customWidth="1"/>
+    <col min="19" max="19" width="40.83203125" customWidth="1"/>
+    <col min="20" max="20" width="33.83203125" customWidth="1"/>
+    <col min="21" max="21" width="20.83203125" customWidth="1"/>
+    <col min="22" max="22" width="17.83203125" customWidth="1"/>
+    <col min="23" max="23" width="12.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -898,27 +883,24 @@
         <v>retencion_rate</v>
       </c>
       <c r="Q1" t="str">
-        <v>quote_document_ref</v>
+        <v>notes</v>
       </c>
       <c r="R1" t="str">
-        <v>notes</v>
+        <v>item_title</v>
       </c>
       <c r="S1" t="str">
-        <v>item_title</v>
+        <v>category</v>
       </c>
       <c r="T1" t="str">
-        <v>category</v>
+        <v>subtotal</v>
       </c>
       <c r="U1" t="str">
-        <v>subtotal</v>
+        <v>quantity</v>
       </c>
       <c r="V1" t="str">
-        <v>quantity</v>
+        <v>unit_of_measure</v>
       </c>
       <c r="W1" t="str">
-        <v>unit_of_measure</v>
-      </c>
-      <c r="X1" t="str">
         <v>unit_price</v>
       </c>
     </row>
@@ -972,27 +954,24 @@
         <v>Retención rate</v>
       </c>
       <c r="Q2" t="str">
-        <v>Linked quote document_ref</v>
+        <v>Notes</v>
       </c>
       <c r="R2" t="str">
-        <v>Notes</v>
+        <v>Line item title</v>
       </c>
       <c r="S2" t="str">
-        <v>Line item title</v>
+        <v>Line item category</v>
       </c>
       <c r="T2" t="str">
-        <v>Line item category</v>
+        <v>Line item subtotal (before IGV)</v>
       </c>
       <c r="U2" t="str">
-        <v>Line item subtotal (before IGV)</v>
+        <v>Line item quantity</v>
       </c>
       <c r="V2" t="str">
-        <v>Line item quantity</v>
+        <v>Unit of measure</v>
       </c>
       <c r="W2" t="str">
-        <v>Unit of measure</v>
-      </c>
-      <c r="X2" t="str">
         <v>Unit price</v>
       </c>
     </row>
@@ -1046,27 +1025,24 @@
         <v>0.03</v>
       </c>
       <c r="Q3" t="str">
-        <v>COT-001</v>
+        <v/>
       </c>
       <c r="R3" t="str">
-        <v/>
+        <v>Cement bags</v>
       </c>
       <c r="S3" t="str">
-        <v>Cement bags</v>
+        <v>materials</v>
       </c>
       <c r="T3" t="str">
-        <v>materials</v>
+        <v>5000.00</v>
       </c>
       <c r="U3" t="str">
-        <v>5000.00</v>
+        <v>200</v>
       </c>
       <c r="V3" t="str">
-        <v>200</v>
+        <v>bags</v>
       </c>
       <c r="W3" t="str">
-        <v>bags</v>
-      </c>
-      <c r="X3" t="str">
         <v>25.00</v>
       </c>
     </row>
@@ -1120,33 +1096,30 @@
         <v/>
       </c>
       <c r="Q4" t="str">
-        <v>Must exist in DB</v>
+        <v/>
       </c>
       <c r="R4" t="str">
         <v/>
       </c>
       <c r="S4" t="str">
-        <v/>
+        <v>materials, labor, subcontractor, equipment_rental, housing_food, other, software_licenses, partner_compensation, professional_services, other_sga</v>
       </c>
       <c r="T4" t="str">
-        <v>materials, labor, subcontractor, equipment_rental, housing_food, other, software_licenses, partner_compensation, professional_services, other_sga</v>
+        <v>Number, &gt; 0</v>
       </c>
       <c r="U4" t="str">
-        <v>Number, &gt; 0</v>
+        <v>Number</v>
       </c>
       <c r="V4" t="str">
-        <v>Number</v>
+        <v/>
       </c>
       <c r="W4" t="str">
-        <v/>
-      </c>
-      <c r="X4" t="str">
         <v>Number</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:X4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: correct rate descriptions in invoice import template
IGV, detraccion, and retencion rate fields now document percentage
values (18, 12, 3) instead of decimal fractions (0.18, 0.12, 0.03).
Added 'pending' to valid comprobante_type values.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/website/public/templates/invoices-template.xlsx
+++ b/website/public/templates/invoices-template.xlsx
@@ -542,10 +542,10 @@
         <v>Yes</v>
       </c>
       <c r="C15" t="str">
-        <v>IGV rate</v>
+        <v>IGV rate (%)</v>
       </c>
       <c r="D15" t="str">
-        <v>0 or 0.18</v>
+        <v>0 or 18</v>
       </c>
     </row>
     <row r="16">
@@ -601,7 +601,7 @@
         <v>Comprobante type</v>
       </c>
       <c r="D19" t="str">
-        <v>factura, boleta, recibo_por_honorarios, liquidacion_de_compra, planilla_jornales, none</v>
+        <v>factura, boleta, recibo_por_honorarios, liquidacion_de_compra, planilla_jornales, none, pending</v>
       </c>
     </row>
     <row r="20">
@@ -640,10 +640,10 @@
         <v>No</v>
       </c>
       <c r="C22" t="str">
-        <v>Detracción rate</v>
+        <v>Detracción rate (%)</v>
       </c>
       <c r="D22" t="str">
-        <v>PEN invoices only</v>
+        <v>0–100, PEN invoices only</v>
       </c>
     </row>
     <row r="23">
@@ -668,10 +668,10 @@
         <v>No</v>
       </c>
       <c r="C24" t="str">
-        <v>Retención rate</v>
+        <v>Retención rate (%)</v>
       </c>
       <c r="D24" t="str">
-        <v/>
+        <v>0–100, receivable only</v>
       </c>
     </row>
     <row r="25">
@@ -814,16 +814,16 @@
     <col min="4" max="4" width="24.83203125" customWidth="1"/>
     <col min="5" max="5" width="16.83203125" customWidth="1"/>
     <col min="6" max="6" width="15.83203125" customWidth="1"/>
-    <col min="7" max="7" width="12.83203125" customWidth="1"/>
+    <col min="7" max="7" width="14.83203125" customWidth="1"/>
     <col min="8" max="8" width="29.83203125" customWidth="1"/>
     <col min="9" max="9" width="18.83203125" customWidth="1"/>
     <col min="10" max="10" width="24.83203125" customWidth="1"/>
     <col min="11" max="11" width="40.83203125" customWidth="1"/>
     <col min="12" max="12" width="35.83203125" customWidth="1"/>
     <col min="13" max="13" width="12.83203125" customWidth="1"/>
-    <col min="14" max="14" width="19.83203125" customWidth="1"/>
+    <col min="14" max="14" width="26.83203125" customWidth="1"/>
     <col min="15" max="15" width="29.83203125" customWidth="1"/>
-    <col min="16" max="16" width="16.83203125" customWidth="1"/>
+    <col min="16" max="16" width="24.83203125" customWidth="1"/>
     <col min="17" max="17" width="12.83203125" customWidth="1"/>
     <col min="18" max="18" width="17.83203125" customWidth="1"/>
     <col min="19" max="19" width="40.83203125" customWidth="1"/>
@@ -924,7 +924,7 @@
         <v>Currency code</v>
       </c>
       <c r="G2" t="str">
-        <v>IGV rate</v>
+        <v>IGV rate (%)</v>
       </c>
       <c r="H2" t="str">
         <v>Exchange rate (PEN per USD)</v>
@@ -945,13 +945,13 @@
         <v>Due date</v>
       </c>
       <c r="N2" t="str">
-        <v>Detracción rate</v>
+        <v>Detracción rate (%)</v>
       </c>
       <c r="O2" t="str">
         <v>Retención applies?</v>
       </c>
       <c r="P2" t="str">
-        <v>Retención rate</v>
+        <v>Retención rate (%)</v>
       </c>
       <c r="Q2" t="str">
         <v>Notes</v>
@@ -995,7 +995,7 @@
         <v>PEN</v>
       </c>
       <c r="G3" t="str">
-        <v>0.18</v>
+        <v>18</v>
       </c>
       <c r="H3" t="str">
         <v>3.72</v>
@@ -1016,13 +1016,13 @@
         <v>2026-04-15</v>
       </c>
       <c r="N3" t="str">
-        <v>0.12</v>
+        <v>12</v>
       </c>
       <c r="O3" t="str">
         <v>false</v>
       </c>
       <c r="P3" t="str">
-        <v>0.03</v>
+        <v>3</v>
       </c>
       <c r="Q3" t="str">
         <v/>
@@ -1066,7 +1066,7 @@
         <v>USD, PEN</v>
       </c>
       <c r="G4" t="str">
-        <v>0 or 0.18</v>
+        <v>0 or 18</v>
       </c>
       <c r="H4" t="str">
         <v>2.5–6.0</v>
@@ -1078,7 +1078,7 @@
         <v>Must exist in DB</v>
       </c>
       <c r="K4" t="str">
-        <v>factura, boleta, recibo_por_honorarios, liquidacion_de_compra, planilla_jornales, none</v>
+        <v>factura, boleta, recibo_por_honorarios, liquidacion_de_compra, planilla_jornales, none, pending</v>
       </c>
       <c r="L4" t="str">
         <v/>
@@ -1087,13 +1087,13 @@
         <v>YYYY-MM-DD</v>
       </c>
       <c r="N4" t="str">
-        <v>PEN invoices only</v>
+        <v>0–100, PEN invoices only</v>
       </c>
       <c r="O4" t="str">
         <v>true/false, receivable only</v>
       </c>
       <c r="P4" t="str">
-        <v/>
+        <v>0–100, receivable only</v>
       </c>
       <c r="Q4" t="str">
         <v/>

</xml_diff>

<commit_message>
chore: regenerate Excel templates after quote lifecycle changes
- Quotes template: add notes about quote lifecycle (pending/rejected invisible
  to financial views, only accepted quotes become real invoices)
- Invoices template: update retencion_rate example to 8%, add auto-default note
- Regenerated all three .xlsx template files

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/website/public/templates/invoices-template.xlsx
+++ b/website/public/templates/invoices-template.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D37"/>
+  <dimension ref="A1:D38"/>
   <cols>
     <col min="1" max="1" width="28.83203125" customWidth="1"/>
     <col min="2" max="2" width="44.83203125" customWidth="1"/>
@@ -668,7 +668,7 @@
         <v>No</v>
       </c>
       <c r="C24" t="str">
-        <v>Retención rate (%)</v>
+        <v>Retención rate (%). Defaults to 8% if retencion_applicable=true</v>
       </c>
       <c r="D24" t="str">
         <v>0–100, receivable only</v>
@@ -797,9 +797,14 @@
         <v xml:space="preserve">  - Retención only applies to receivable invoices</v>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v xml:space="preserve">  - If retencion_applicable=true and no retencion_rate is provided, defaults to 8%</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D37"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D38"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -823,7 +828,7 @@
     <col min="13" max="13" width="12.83203125" customWidth="1"/>
     <col min="14" max="14" width="26.83203125" customWidth="1"/>
     <col min="15" max="15" width="29.83203125" customWidth="1"/>
-    <col min="16" max="16" width="24.83203125" customWidth="1"/>
+    <col min="16" max="16" width="40.83203125" customWidth="1"/>
     <col min="17" max="17" width="12.83203125" customWidth="1"/>
     <col min="18" max="18" width="17.83203125" customWidth="1"/>
     <col min="19" max="19" width="40.83203125" customWidth="1"/>
@@ -951,7 +956,7 @@
         <v>Retención applies?</v>
       </c>
       <c r="P2" t="str">
-        <v>Retención rate (%)</v>
+        <v>Retención rate (%). Defaults to 8% if retencion_applicable=true</v>
       </c>
       <c r="Q2" t="str">
         <v>Notes</v>
@@ -1022,7 +1027,7 @@
         <v>false</v>
       </c>
       <c r="P3" t="str">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="Q3" t="str">
         <v/>

</xml_diff>